<commit_message>
Add scripts for consolidating and reporting supplier data
- Introduced `consolidar_pepsico.py` to consolidate quarterly purchases from PEPSICO into a single Excel file, optimizing memory usage and handling large datasets efficiently.
- Created `gen_plan_ejecucion.py` to define which suppliers to execute based on planning data, generating a detailed execution plan in Excel format.
- Developed `reporte_cruce.py` to generate structured reports on CPA Vision to Purchases metrics, allowing for analysis of supplier performance and EDI coverage.
- Added a new CSV file `rfc_por_proveedor.csv` containing supplier RFCs for reference in the new scripts.
</commit_message>
<xml_diff>
--- a/descarga_monica_pendientes.xlsx
+++ b/descarga_monica_pendientes.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="67">
   <si>
     <t>RFC</t>
   </si>
@@ -31,66 +31,9 @@
     <t>Prioridad</t>
   </si>
   <si>
-    <t>IOT180425UE9</t>
-  </si>
-  <si>
     <t>IGU880227Q96</t>
   </si>
   <si>
-    <t>SIB080429PG5</t>
-  </si>
-  <si>
-    <t>PIP1309236AA</t>
-  </si>
-  <si>
-    <t>MSH970109JX2</t>
-  </si>
-  <si>
-    <t>GDA861201JL8</t>
-  </si>
-  <si>
-    <t>CIN860808CQA</t>
-  </si>
-  <si>
-    <t>HMP980506HD0</t>
-  </si>
-  <si>
-    <t>HTE150424K14</t>
-  </si>
-  <si>
-    <t>GVE990302IH9</t>
-  </si>
-  <si>
-    <t>MCT891212I87</t>
-  </si>
-  <si>
-    <t>DME010612B53</t>
-  </si>
-  <si>
-    <t>AAP111202148</t>
-  </si>
-  <si>
-    <t>SIC881013DX5</t>
-  </si>
-  <si>
-    <t>ARE960611NX4</t>
-  </si>
-  <si>
-    <t>EFR870619KD1</t>
-  </si>
-  <si>
-    <t>CGM130918U80</t>
-  </si>
-  <si>
-    <t>DDE720607UI7</t>
-  </si>
-  <si>
-    <t>VVA851125PF6</t>
-  </si>
-  <si>
-    <t>MPM120821CNA</t>
-  </si>
-  <si>
     <t>DPI120830A78</t>
   </si>
   <si>
@@ -160,42 +103,30 @@
     <t>SMA011011BQ5</t>
   </si>
   <si>
-    <t>2022 2023 2025</t>
-  </si>
-  <si>
     <t>2023</t>
   </si>
   <si>
     <t>2021 2022 2023</t>
   </si>
   <si>
-    <t>2020 2021 2022 2023 2025</t>
+    <t>2021 2022</t>
+  </si>
+  <si>
+    <t>2021</t>
+  </si>
+  <si>
+    <t>2020 2021</t>
+  </si>
+  <si>
+    <t>2022</t>
+  </si>
+  <si>
+    <t>2024</t>
   </si>
   <si>
     <t>2025</t>
   </si>
   <si>
-    <t>2020 2021</t>
-  </si>
-  <si>
-    <t>2021 2022 2024</t>
-  </si>
-  <si>
-    <t>2022 2023 2024</t>
-  </si>
-  <si>
-    <t>2021 2022</t>
-  </si>
-  <si>
-    <t>2021</t>
-  </si>
-  <si>
-    <t>2022</t>
-  </si>
-  <si>
-    <t>2024</t>
-  </si>
-  <si>
     <t>2023 2025</t>
   </si>
   <si>
@@ -214,64 +145,7 @@
     <t>2022 2025</t>
   </si>
   <si>
-    <t>IOTZONE SA DE CV</t>
-  </si>
-  <si>
     <t>INDUSTRIAS GUACAMAYA SA DE CV</t>
-  </si>
-  <si>
-    <t>SKN IMAGEN Y BELLEZA S.A. DE C.V.</t>
-  </si>
-  <si>
-    <t>PANIFICADORA INTEGRAL PLF SA DE CV</t>
-  </si>
-  <si>
-    <t>MEXPROUD SHIPPING SA DE CV</t>
-  </si>
-  <si>
-    <t>GRUPO DAFNA S A DE C V</t>
-  </si>
-  <si>
-    <t>CINSA SA DE CV</t>
-  </si>
-  <si>
-    <t>HORTALIZAS Y MELONES DE PAILA SPR DE R.L.</t>
-  </si>
-  <si>
-    <t>HAPPY TEE SA DE CV</t>
-  </si>
-  <si>
-    <t>GRUPO VERMEX SA DE CV</t>
-  </si>
-  <si>
-    <t>MODA Y CONFECCION TEXTIL PLANETA, S .A. DE C.V.</t>
-  </si>
-  <si>
-    <t>DKT DE MEXICO SA DE CV</t>
-  </si>
-  <si>
-    <t>ALIMENTOS AL PUNTO SA DE CV</t>
-  </si>
-  <si>
-    <t>SERVICIOS INTERNACIONALES DE COMERC IO SA DE CV</t>
-  </si>
-  <si>
-    <t>ARENA Y COMPA¥IA SA DE CV</t>
-  </si>
-  <si>
-    <t>EMPACADORA EL FRESNO S.A. DE C.V.</t>
-  </si>
-  <si>
-    <t>COHEVI GLOBAL MARKET SA DE CV</t>
-  </si>
-  <si>
-    <t>DATILERA DEL DESIERTO S DE RL DE CV</t>
-  </si>
-  <si>
-    <t>VITIVINICOLA VALBUENA SA DE CV</t>
-  </si>
-  <si>
-    <t>MERCANTIL DE PRODUCTOS MORELOS SA DE CV</t>
   </si>
   <si>
     <t>DISTRIBUCIONES PICACHOS SA DE CV</t>
@@ -672,7 +546,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -697,16 +571,16 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="C2">
-        <v>21102</v>
+        <v>44586</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="E2">
-        <v>568</v>
+        <v>595</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -714,16 +588,16 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="C3">
-        <v>44586</v>
+        <v>779</v>
       </c>
       <c r="D3" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E3">
-        <v>595</v>
+        <v>726</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -731,16 +605,16 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="C4">
-        <v>391961</v>
+        <v>22689</v>
       </c>
       <c r="D4" t="s">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="E4">
-        <v>604</v>
+        <v>728</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -748,16 +622,16 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="C5">
-        <v>4437</v>
+        <v>77867</v>
       </c>
       <c r="D5" t="s">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="E5">
-        <v>631</v>
+        <v>729</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -765,16 +639,16 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="C6">
-        <v>23231</v>
+        <v>82289</v>
       </c>
       <c r="D6" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E6">
-        <v>657</v>
+        <v>730</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -782,16 +656,16 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="C7">
-        <v>60699</v>
+        <v>20486</v>
       </c>
       <c r="D7" t="s">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="E7">
-        <v>676</v>
+        <v>734</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -799,16 +673,16 @@
         <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="C8">
-        <v>55004</v>
+        <v>1048</v>
       </c>
       <c r="D8" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="E8">
-        <v>681</v>
+        <v>735</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -816,16 +690,16 @@
         <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="C9">
-        <v>323618</v>
+        <v>24388</v>
       </c>
       <c r="D9" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="E9">
-        <v>685</v>
+        <v>736</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -833,16 +707,16 @@
         <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="C10">
-        <v>22225</v>
+        <v>21930</v>
       </c>
       <c r="D10" t="s">
-        <v>74</v>
+        <v>51</v>
       </c>
       <c r="E10">
-        <v>687</v>
+        <v>739</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -850,16 +724,16 @@
         <v>14</v>
       </c>
       <c r="B11" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="C11">
-        <v>380220</v>
+        <v>24072</v>
       </c>
       <c r="D11" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="E11">
-        <v>690</v>
+        <v>740</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -867,16 +741,16 @@
         <v>15</v>
       </c>
       <c r="B12" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="C12">
-        <v>1966</v>
+        <v>2121</v>
       </c>
       <c r="D12" t="s">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="E12">
-        <v>696</v>
+        <v>741</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -884,16 +758,16 @@
         <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="C13">
-        <v>318493</v>
+        <v>68494</v>
       </c>
       <c r="D13" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
       <c r="E13">
-        <v>705</v>
+        <v>744</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -901,16 +775,16 @@
         <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="C14">
-        <v>1814</v>
+        <v>395434</v>
       </c>
       <c r="D14" t="s">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="E14">
-        <v>706</v>
+        <v>745</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -918,16 +792,16 @@
         <v>18</v>
       </c>
       <c r="B15" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="C15">
-        <v>378562</v>
+        <v>384578</v>
       </c>
       <c r="D15" t="s">
-        <v>79</v>
+        <v>56</v>
       </c>
       <c r="E15">
-        <v>708</v>
+        <v>746</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -935,16 +809,16 @@
         <v>19</v>
       </c>
       <c r="B16" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="C16">
-        <v>23939</v>
+        <v>23789</v>
       </c>
       <c r="D16" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="E16">
-        <v>712</v>
+        <v>747</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -952,16 +826,16 @@
         <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="C17">
-        <v>15191</v>
+        <v>96685</v>
       </c>
       <c r="D17" t="s">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="E17">
-        <v>713</v>
+        <v>748</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -969,16 +843,16 @@
         <v>21</v>
       </c>
       <c r="B18" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C18">
-        <v>9264</v>
+        <v>314658</v>
       </c>
       <c r="D18" t="s">
-        <v>82</v>
+        <v>59</v>
       </c>
       <c r="E18">
-        <v>715</v>
+        <v>749</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -986,16 +860,16 @@
         <v>22</v>
       </c>
       <c r="B19" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="C19">
-        <v>41988</v>
+        <v>312132</v>
       </c>
       <c r="D19" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="E19">
-        <v>718</v>
+        <v>750</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -1003,16 +877,16 @@
         <v>23</v>
       </c>
       <c r="B20" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="C20">
-        <v>23652</v>
+        <v>23744</v>
       </c>
       <c r="D20" t="s">
-        <v>84</v>
+        <v>61</v>
       </c>
       <c r="E20">
-        <v>720</v>
+        <v>751</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -1020,16 +894,16 @@
         <v>24</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="C21">
-        <v>10948</v>
+        <v>250148</v>
       </c>
       <c r="D21" t="s">
-        <v>85</v>
+        <v>62</v>
       </c>
       <c r="E21">
-        <v>725</v>
+        <v>753</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -1037,16 +911,16 @@
         <v>25</v>
       </c>
       <c r="B22" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="C22">
-        <v>779</v>
+        <v>303428</v>
       </c>
       <c r="D22" t="s">
-        <v>86</v>
+        <v>63</v>
       </c>
       <c r="E22">
-        <v>726</v>
+        <v>756</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -1054,16 +928,16 @@
         <v>26</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="C23">
-        <v>22689</v>
+        <v>394403</v>
       </c>
       <c r="D23" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
       <c r="E23">
-        <v>728</v>
+        <v>758</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -1071,16 +945,16 @@
         <v>27</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>36</v>
       </c>
       <c r="C24">
-        <v>77867</v>
+        <v>64675</v>
       </c>
       <c r="D24" t="s">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="E24">
-        <v>729</v>
+        <v>759</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1088,338 +962,15 @@
         <v>28</v>
       </c>
       <c r="B25" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="C25">
-        <v>82289</v>
+        <v>308619</v>
       </c>
       <c r="D25" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="E25">
-        <v>730</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="A26" t="s">
-        <v>29</v>
-      </c>
-      <c r="B26" t="s">
-        <v>58</v>
-      </c>
-      <c r="C26">
-        <v>20486</v>
-      </c>
-      <c r="D26" t="s">
-        <v>90</v>
-      </c>
-      <c r="E26">
-        <v>734</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="A27" t="s">
-        <v>30</v>
-      </c>
-      <c r="B27" t="s">
-        <v>59</v>
-      </c>
-      <c r="C27">
-        <v>1048</v>
-      </c>
-      <c r="D27" t="s">
-        <v>91</v>
-      </c>
-      <c r="E27">
-        <v>735</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5">
-      <c r="A28" t="s">
-        <v>31</v>
-      </c>
-      <c r="B28" t="s">
-        <v>52</v>
-      </c>
-      <c r="C28">
-        <v>24388</v>
-      </c>
-      <c r="D28" t="s">
-        <v>92</v>
-      </c>
-      <c r="E28">
-        <v>736</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5">
-      <c r="A29" t="s">
-        <v>32</v>
-      </c>
-      <c r="B29" t="s">
-        <v>59</v>
-      </c>
-      <c r="C29">
-        <v>21930</v>
-      </c>
-      <c r="D29" t="s">
-        <v>93</v>
-      </c>
-      <c r="E29">
-        <v>739</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5">
-      <c r="A30" t="s">
-        <v>33</v>
-      </c>
-      <c r="B30" t="s">
-        <v>52</v>
-      </c>
-      <c r="C30">
-        <v>24072</v>
-      </c>
-      <c r="D30" t="s">
-        <v>94</v>
-      </c>
-      <c r="E30">
-        <v>740</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5">
-      <c r="A31" t="s">
-        <v>34</v>
-      </c>
-      <c r="B31" t="s">
-        <v>52</v>
-      </c>
-      <c r="C31">
-        <v>2121</v>
-      </c>
-      <c r="D31" t="s">
-        <v>95</v>
-      </c>
-      <c r="E31">
-        <v>741</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5">
-      <c r="A32" t="s">
-        <v>35</v>
-      </c>
-      <c r="B32" t="s">
-        <v>60</v>
-      </c>
-      <c r="C32">
-        <v>68494</v>
-      </c>
-      <c r="D32" t="s">
-        <v>96</v>
-      </c>
-      <c r="E32">
-        <v>744</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5">
-      <c r="A33" t="s">
-        <v>36</v>
-      </c>
-      <c r="B33" t="s">
-        <v>61</v>
-      </c>
-      <c r="C33">
-        <v>395434</v>
-      </c>
-      <c r="D33" t="s">
-        <v>97</v>
-      </c>
-      <c r="E33">
-        <v>745</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5">
-      <c r="A34" t="s">
-        <v>37</v>
-      </c>
-      <c r="B34" t="s">
-        <v>62</v>
-      </c>
-      <c r="C34">
-        <v>384578</v>
-      </c>
-      <c r="D34" t="s">
-        <v>98</v>
-      </c>
-      <c r="E34">
-        <v>746</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5">
-      <c r="A35" t="s">
-        <v>38</v>
-      </c>
-      <c r="B35" t="s">
-        <v>52</v>
-      </c>
-      <c r="C35">
-        <v>23789</v>
-      </c>
-      <c r="D35" t="s">
-        <v>99</v>
-      </c>
-      <c r="E35">
-        <v>747</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5">
-      <c r="A36" t="s">
-        <v>39</v>
-      </c>
-      <c r="B36" t="s">
-        <v>50</v>
-      </c>
-      <c r="C36">
-        <v>96685</v>
-      </c>
-      <c r="D36" t="s">
-        <v>100</v>
-      </c>
-      <c r="E36">
-        <v>748</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5">
-      <c r="A37" t="s">
-        <v>40</v>
-      </c>
-      <c r="B37" t="s">
-        <v>63</v>
-      </c>
-      <c r="C37">
-        <v>314658</v>
-      </c>
-      <c r="D37" t="s">
-        <v>101</v>
-      </c>
-      <c r="E37">
-        <v>749</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5">
-      <c r="A38" t="s">
-        <v>41</v>
-      </c>
-      <c r="B38" t="s">
-        <v>64</v>
-      </c>
-      <c r="C38">
-        <v>312132</v>
-      </c>
-      <c r="D38" t="s">
-        <v>102</v>
-      </c>
-      <c r="E38">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5">
-      <c r="A39" t="s">
-        <v>42</v>
-      </c>
-      <c r="B39" t="s">
-        <v>65</v>
-      </c>
-      <c r="C39">
-        <v>23744</v>
-      </c>
-      <c r="D39" t="s">
-        <v>103</v>
-      </c>
-      <c r="E39">
-        <v>751</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5">
-      <c r="A40" t="s">
-        <v>43</v>
-      </c>
-      <c r="B40" t="s">
-        <v>65</v>
-      </c>
-      <c r="C40">
-        <v>250148</v>
-      </c>
-      <c r="D40" t="s">
-        <v>104</v>
-      </c>
-      <c r="E40">
-        <v>753</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5">
-      <c r="A41" t="s">
-        <v>44</v>
-      </c>
-      <c r="B41" t="s">
-        <v>53</v>
-      </c>
-      <c r="C41">
-        <v>303428</v>
-      </c>
-      <c r="D41" t="s">
-        <v>105</v>
-      </c>
-      <c r="E41">
-        <v>756</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5">
-      <c r="A42" t="s">
-        <v>45</v>
-      </c>
-      <c r="B42" t="s">
-        <v>56</v>
-      </c>
-      <c r="C42">
-        <v>394403</v>
-      </c>
-      <c r="D42" t="s">
-        <v>106</v>
-      </c>
-      <c r="E42">
-        <v>758</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5">
-      <c r="A43" t="s">
-        <v>46</v>
-      </c>
-      <c r="B43" t="s">
-        <v>52</v>
-      </c>
-      <c r="C43">
-        <v>64675</v>
-      </c>
-      <c r="D43" t="s">
-        <v>107</v>
-      </c>
-      <c r="E43">
-        <v>759</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5">
-      <c r="A44" t="s">
-        <v>47</v>
-      </c>
-      <c r="B44" t="s">
-        <v>52</v>
-      </c>
-      <c r="C44">
-        <v>308619</v>
-      </c>
-      <c r="D44" t="s">
-        <v>108</v>
-      </c>
-      <c r="E44">
         <v>760</v>
       </c>
     </row>

</xml_diff>